<commit_message>
Update Stoned Build Change Logs.xlsx
</commit_message>
<xml_diff>
--- a/Docs/Stoned Build Change Logs.xlsx
+++ b/Docs/Stoned Build Change Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shield\Documents\Unity\Stonicorn\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78274A5C-7D93-429F-A995-B46DBCBFAB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984876D3-3DE0-4808-A292-5C5B5425A006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19260" yWindow="6450" windowWidth="20475" windowHeight="12570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24090" yWindow="6180" windowWidth="17340" windowHeight="13425" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Builds" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="886">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="887">
   <si>
     <t>Stoned Builds Change Log</t>
   </si>
@@ -2699,6 +2699,9 @@
   </si>
   <si>
     <t>#620, #629</t>
+  </si>
+  <si>
+    <t>0.603</t>
   </si>
 </sst>
 </file>
@@ -7816,7 +7819,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923D1F1C-9339-49C8-9FCA-FF86526676FD}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A3:G45"/>
+  <dimension ref="A3:G46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -8722,6 +8725,26 @@
       </c>
       <c r="F45" s="9">
         <v>1.4694444444444446</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="6">
+        <v>45692</v>
+      </c>
+      <c r="B46" s="10">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>886</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>743</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>724</v>
+      </c>
+      <c r="F46" s="9">
+        <v>1.3805555555555555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>